<commit_message>
added tex file for report
</commit_message>
<xml_diff>
--- a/port_vs_nifty_analysis_details.xlsx
+++ b/port_vs_nifty_analysis_details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1f0000be4cca5a50/MFE tasks/Capstone project/Project_code/WQU_Capstone_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{1C915199-FB21-8D45-B835-30859C11EA32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4FEAA49-7A2A-A040-8BDC-2250F9A7C03A}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{1C915199-FB21-8D45-B835-30859C11EA32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E77F6AE-EDF6-1649-B086-8B9624FB43F0}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="480" windowWidth="28800" windowHeight="17520" xr2:uid="{E26E1912-ED3F-BB41-BAA9-752401DFEDE6}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16180" xr2:uid="{E26E1912-ED3F-BB41-BAA9-752401DFEDE6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
     <t>NIFTY50</t>
   </si>
   <si>
-    <t>Month End Date</t>
+    <t>Month_End</t>
   </si>
 </sst>
 </file>
@@ -199,185 +199,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8782013-6713-FBF5-E254-DC77DFA570C2}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="15278100" y="0"/>
-          <a:ext cx="7543800" cy="3746500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4DA4FA9-E26D-34EC-E52B-CF8EA32693DC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="15278100" y="4457700"/>
-          <a:ext cx="7543800" cy="3746500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>65329</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD43A366-70C9-5A94-6FAC-0851BEC723A7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="15278100" y="9029700"/>
-          <a:ext cx="7772400" cy="3303829"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C68B323A-C542-9D28-C226-B568302EF98A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="15278100" y="12649200"/>
-          <a:ext cx="7543800" cy="3746500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5278,6 +5101,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>